<commit_message>
fix: improve port matching, STS duration calculation, and add duplicate detection
- Add new port name variants (zhoushaneast, xiazhimensouth, north anchorage, qushanbun)
- Add "Broken Up" vessel status to regex pattern
- Fix STS duration to use raw timestamps instead of rounded ones
- Fix end_STS_final to use last STS slot instead of max end time
- Add transaction-level duplicate detection with logging
- Replace Python matching scripts with Stata .do files
- Remove run_all.sh and old HTML doc
</commit_message>
<xml_diff>
--- a/logs/duplicate_records.xlsx
+++ b/logs/duplicate_records.xlsx
@@ -4833,7 +4833,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>SERENITY 1 (9060247) - Bulk Carrier, Broken Up, 28458 dwt, 17430gt</t>
+          <t>SERENITY 1</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>SERENITY 1 (9060247) - Bulk Carrier, Broken Up, 28458 dwt, 17430gt</t>
+          <t>SERENITY 1</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>SERENITY 1 (9060247) - Bulk Carrier, Broken Up, 28458 dwt, 17430gt</t>
+          <t>SERENITY 1</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>SERENITY 1 (9060247) - Bulk Carrier, Broken Up, 28458 dwt, 17430gt</t>
+          <t>SERENITY 1</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>SERENITY 1 (9060247) - Bulk Carrier, Broken Up, 28458 dwt, 17430gt</t>
+          <t>SERENITY 1</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>SERENITY 1 (9060247) - Bulk Carrier, Broken Up, 28458 dwt, 17430gt</t>
+          <t>SERENITY 1</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>SERENITY 1 (9060247) - Bulk Carrier, Broken Up, 28458 dwt, 17430gt</t>
+          <t>SERENITY 1</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>SERENITY 1 (9060247) - Bulk Carrier, Broken Up, 28458 dwt, 17430gt</t>
+          <t>SERENITY 1</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -5355,7 +5355,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>RADA (9213301) - Crude Oil Tanker, Broken Up, 112201 dwt, 62385gt</t>
+          <t>RADA</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -5384,7 +5384,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>RADA (9213301) - Crude Oil Tanker, Broken Up, 112201 dwt, 62385gt</t>
+          <t>RADA</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -5413,7 +5413,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>RADA (9213301) - Crude Oil Tanker, Broken Up, 112201 dwt, 62385gt</t>
+          <t>RADA</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>RADA (9213301) - Crude Oil Tanker, Broken Up, 112201 dwt, 62385gt</t>
+          <t>RADA</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -5471,7 +5471,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>RADA (9213301) - Crude Oil Tanker, Broken Up, 112201 dwt, 62385gt</t>
+          <t>RADA</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>RADA (9213301) - Crude Oil Tanker, Broken Up, 112201 dwt, 62385gt</t>
+          <t>RADA</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">

</xml_diff>